<commit_message>
Update Shacman X5000 prices: 5.89M→6.09M, 5.69M→5.99M
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018DCThKeZxZvYg85WAqJNLy
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -839,7 +839,7 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>5890000</t>
+          <t>6090000</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr"/>
@@ -918,7 +918,7 @@
       <c r="AH2" s="1" t="inlineStr"/>
       <c r="AI2" s="1" t="inlineStr">
         <is>
-          <t>5890000</t>
+          <t>6090000</t>
         </is>
       </c>
       <c r="AJ2" s="1" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="L3" s="1" t="inlineStr">
         <is>
-          <t>5690000</t>
+          <t>5990000</t>
         </is>
       </c>
       <c r="M3" s="1" t="inlineStr"/>
@@ -1117,7 +1117,7 @@
       <c r="AH3" s="1" t="inlineStr"/>
       <c r="AI3" s="1" t="inlineStr">
         <is>
-          <t>5690000</t>
+          <t>5990000</t>
         </is>
       </c>
       <c r="AJ3" s="1" t="inlineStr">

</xml_diff>

<commit_message>
B-Trailer: Shacman X5000 ×2 (rx065529, rx065530) проданы — сняты из фида
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK3"/>
+  <dimension ref="A1:BK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -425,19 +425,19 @@
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="28" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="10" customWidth="1" min="24" max="24"/>
@@ -462,7 +462,7 @@
     <col width="33" customWidth="1" min="43" max="43"/>
     <col width="10" customWidth="1" min="44" max="44"/>
     <col width="16" customWidth="1" min="45" max="45"/>
-    <col width="12" customWidth="1" min="46" max="46"/>
+    <col width="11" customWidth="1" min="46" max="46"/>
     <col width="10" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="10" customWidth="1" min="49" max="49"/>
@@ -799,430 +799,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>shacman-x5000-rx065529</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr"/>
-      <c r="C2" s="1" t="inlineStr"/>
-      <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr"/>
-      <c r="F2" s="1" t="inlineStr"/>
-      <c r="G2" s="1" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>79685590315</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>По телефону и в сообщениях</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>Самосвал Shacman X5000, 2024 год выпуска.
-Двигатель WP12.550E50, 550 л.с., дизель, объём 11 596 см³, 6 цилиндров, крутящий момент 2060 Н·м, экологический класс Евро 5.
-Колёсная формула 8×4, коробка механическая, 12 передач.
-Пробег 93 293 км, техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
-Кузов — самосвал, объём 35 м³ (35000 л).
-Снаряжённая масса 19 500 кг, разрешённая максимальная масса 60 500 кг, грузоподъёмность 41 000 кг.
-Объём топливного бака 500 л, максимальная скорость 80 км/ч.
-Шины 315/80R22.5 (перед/зад).
-Страна происхождения — Китай.
-Документы в порядке. Смотровая площадка и показ — по договорённости.
-Торг при осмотре.
-Возможна покупка в лизинг через партнёров: Европлан, ВТБ Лизинг, Сберлизинг, Газпромбанк Лизинг, РЕСО Лизинг и др.</t>
-        </is>
-      </c>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>Грузовики и спецтехника</t>
-        </is>
-      </c>
-      <c r="L2" s="1" t="inlineStr">
-        <is>
-          <t>6090000</t>
-        </is>
-      </c>
-      <c r="M2" s="1" t="inlineStr"/>
-      <c r="N2" s="1" t="inlineStr"/>
-      <c r="O2" s="1" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/10.jpg</t>
-        </is>
-      </c>
-      <c r="P2" s="1" t="inlineStr"/>
-      <c r="Q2" s="1" t="inlineStr">
-        <is>
-          <t>Москва, Ижорская ул., 15с2</t>
-        </is>
-      </c>
-      <c r="R2" s="1" t="inlineStr">
-        <is>
-          <t>55.8958019</t>
-        </is>
-      </c>
-      <c r="S2" s="1" t="inlineStr">
-        <is>
-          <t>37.5237956</t>
-        </is>
-      </c>
-      <c r="T2" s="1" t="inlineStr"/>
-      <c r="U2" s="1" t="inlineStr">
-        <is>
-          <t>Москва, Ижорская ул., 15с2</t>
-        </is>
-      </c>
-      <c r="V2" s="1" t="inlineStr">
-        <is>
-          <t>Shacman</t>
-        </is>
-      </c>
-      <c r="W2" s="1" t="inlineStr">
-        <is>
-          <t>Самосвал</t>
-        </is>
-      </c>
-      <c r="X2" s="1" t="inlineStr">
-        <is>
-          <t>X5000</t>
-        </is>
-      </c>
-      <c r="Y2" s="1" t="inlineStr">
-        <is>
-          <t>8×4</t>
-        </is>
-      </c>
-      <c r="Z2" s="1" t="inlineStr">
-        <is>
-          <t>Дизель</t>
-        </is>
-      </c>
-      <c r="AA2" s="1" t="inlineStr">
-        <is>
-          <t>550</t>
-        </is>
-      </c>
-      <c r="AB2" s="1" t="inlineStr">
-        <is>
-          <t>Механика</t>
-        </is>
-      </c>
-      <c r="AC2" s="1" t="inlineStr"/>
-      <c r="AD2" s="1" t="inlineStr"/>
-      <c r="AE2" s="1" t="inlineStr">
-        <is>
-          <t>Грузовики</t>
-        </is>
-      </c>
-      <c r="AF2" s="1" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="AG2" s="1" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="AH2" s="1" t="inlineStr"/>
-      <c r="AI2" s="1" t="inlineStr">
-        <is>
-          <t>6090000</t>
-        </is>
-      </c>
-      <c r="AJ2" s="1" t="inlineStr">
-        <is>
-          <t>Под заказ</t>
-        </is>
-      </c>
-      <c r="AK2" s="1" t="inlineStr"/>
-      <c r="AL2" s="1" t="inlineStr"/>
-      <c r="AM2" s="1" t="inlineStr"/>
-      <c r="AN2" s="1" t="inlineStr"/>
-      <c r="AO2" s="1" t="inlineStr"/>
-      <c r="AP2" s="1" t="inlineStr"/>
-      <c r="AQ2" s="1" t="inlineStr"/>
-      <c r="AR2" s="1" t="inlineStr"/>
-      <c r="AS2" s="1" t="inlineStr"/>
-      <c r="AT2" s="1" t="inlineStr">
-        <is>
-          <t>С пробегом</t>
-        </is>
-      </c>
-      <c r="AU2" s="1" t="inlineStr">
-        <is>
-          <t>93293</t>
-        </is>
-      </c>
-      <c r="AV2" s="1" t="inlineStr">
-        <is>
-          <t>В наличии</t>
-        </is>
-      </c>
-      <c r="AW2" s="1" t="inlineStr"/>
-      <c r="AX2" s="1" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="AY2" s="1" t="inlineStr"/>
-      <c r="AZ2" s="1" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="BA2" s="1" t="inlineStr"/>
-      <c r="BB2" s="1" t="inlineStr"/>
-      <c r="BC2" s="1" t="inlineStr"/>
-      <c r="BD2" s="1" t="inlineStr"/>
-      <c r="BE2" s="1" t="inlineStr"/>
-      <c r="BF2" s="1" t="inlineStr">
-        <is>
-          <t>LZGJX4Z6XRX065529</t>
-        </is>
-      </c>
-      <c r="BG2" s="1" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="BH2" s="1" t="inlineStr">
-        <is>
-          <t>41000</t>
-        </is>
-      </c>
-      <c r="BI2" s="1" t="inlineStr">
-        <is>
-          <t>60500</t>
-        </is>
-      </c>
-      <c r="BJ2" s="1" t="inlineStr">
-        <is>
-          <t>11596</t>
-        </is>
-      </c>
-      <c r="BK2" s="1" t="inlineStr">
-        <is>
-          <t>Евро 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>shacman-x5000-rx065530</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr"/>
-      <c r="C3" s="1" t="inlineStr"/>
-      <c r="D3" s="1" t="inlineStr"/>
-      <c r="E3" s="1" t="inlineStr"/>
-      <c r="F3" s="1" t="inlineStr"/>
-      <c r="G3" s="1" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>79685590315</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>По телефону и в сообщениях</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="inlineStr">
-        <is>
-          <t>Самосвал Shacman X5000, 2024 год выпуска.
-Двигатель WP12.550E50, 550 л.с., дизель, объём 11 596 см³, 6 цилиндров, крутящий момент 2060 Н·м, экологический класс Евро 5.
-Колёсная формула 8×4, коробка механическая, 12 передач.
-Пробег 97 616 км, техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
-Кузов — самосвал, объём 35 м³ (35000 л).
-Снаряжённая масса 19 500 кг, разрешённая максимальная масса 60 500 кг, грузоподъёмность 41 000 кг.
-Объём топливного бака 500 л, максимальная скорость 80 км/ч.
-Шины 315/80R22.5 (перед/зад).
-Страна происхождения — Китай.
-Документы в порядке. Смотровая площадка и показ — по договорённости.
-Торг при осмотре.
-Возможна покупка в лизинг через партнёров: Европлан, ВТБ Лизинг, Сберлизинг, Газпромбанк Лизинг, РЕСО Лизинг и др.</t>
-        </is>
-      </c>
-      <c r="K3" s="1" t="inlineStr">
-        <is>
-          <t>Грузовики и спецтехника</t>
-        </is>
-      </c>
-      <c r="L3" s="1" t="inlineStr">
-        <is>
-          <t>5990000</t>
-        </is>
-      </c>
-      <c r="M3" s="1" t="inlineStr"/>
-      <c r="N3" s="1" t="inlineStr"/>
-      <c r="O3" s="1" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/09.jpg</t>
-        </is>
-      </c>
-      <c r="P3" s="1" t="inlineStr"/>
-      <c r="Q3" s="1" t="inlineStr">
-        <is>
-          <t>Москва, Ижорская ул., 15с2</t>
-        </is>
-      </c>
-      <c r="R3" s="1" t="inlineStr">
-        <is>
-          <t>55.8958019</t>
-        </is>
-      </c>
-      <c r="S3" s="1" t="inlineStr">
-        <is>
-          <t>37.5237956</t>
-        </is>
-      </c>
-      <c r="T3" s="1" t="inlineStr"/>
-      <c r="U3" s="1" t="inlineStr">
-        <is>
-          <t>Москва, Ижорская ул., 15с2</t>
-        </is>
-      </c>
-      <c r="V3" s="1" t="inlineStr">
-        <is>
-          <t>Shacman</t>
-        </is>
-      </c>
-      <c r="W3" s="1" t="inlineStr">
-        <is>
-          <t>Самосвал</t>
-        </is>
-      </c>
-      <c r="X3" s="1" t="inlineStr">
-        <is>
-          <t>X5000</t>
-        </is>
-      </c>
-      <c r="Y3" s="1" t="inlineStr">
-        <is>
-          <t>8×4</t>
-        </is>
-      </c>
-      <c r="Z3" s="1" t="inlineStr">
-        <is>
-          <t>Дизель</t>
-        </is>
-      </c>
-      <c r="AA3" s="1" t="inlineStr">
-        <is>
-          <t>550</t>
-        </is>
-      </c>
-      <c r="AB3" s="1" t="inlineStr">
-        <is>
-          <t>Механика</t>
-        </is>
-      </c>
-      <c r="AC3" s="1" t="inlineStr"/>
-      <c r="AD3" s="1" t="inlineStr"/>
-      <c r="AE3" s="1" t="inlineStr">
-        <is>
-          <t>Грузовики</t>
-        </is>
-      </c>
-      <c r="AF3" s="1" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="AG3" s="1" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="AH3" s="1" t="inlineStr"/>
-      <c r="AI3" s="1" t="inlineStr">
-        <is>
-          <t>5990000</t>
-        </is>
-      </c>
-      <c r="AJ3" s="1" t="inlineStr">
-        <is>
-          <t>Под заказ</t>
-        </is>
-      </c>
-      <c r="AK3" s="1" t="inlineStr"/>
-      <c r="AL3" s="1" t="inlineStr"/>
-      <c r="AM3" s="1" t="inlineStr"/>
-      <c r="AN3" s="1" t="inlineStr"/>
-      <c r="AO3" s="1" t="inlineStr"/>
-      <c r="AP3" s="1" t="inlineStr"/>
-      <c r="AQ3" s="1" t="inlineStr"/>
-      <c r="AR3" s="1" t="inlineStr"/>
-      <c r="AS3" s="1" t="inlineStr"/>
-      <c r="AT3" s="1" t="inlineStr">
-        <is>
-          <t>С пробегом</t>
-        </is>
-      </c>
-      <c r="AU3" s="1" t="inlineStr">
-        <is>
-          <t>97616</t>
-        </is>
-      </c>
-      <c r="AV3" s="1" t="inlineStr">
-        <is>
-          <t>В наличии</t>
-        </is>
-      </c>
-      <c r="AW3" s="1" t="inlineStr"/>
-      <c r="AX3" s="1" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="AY3" s="1" t="inlineStr"/>
-      <c r="AZ3" s="1" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="BA3" s="1" t="inlineStr"/>
-      <c r="BB3" s="1" t="inlineStr"/>
-      <c r="BC3" s="1" t="inlineStr"/>
-      <c r="BD3" s="1" t="inlineStr"/>
-      <c r="BE3" s="1" t="inlineStr"/>
-      <c r="BF3" s="1" t="inlineStr">
-        <is>
-          <t>LZGJX4Z66RX065530</t>
-        </is>
-      </c>
-      <c r="BG3" s="1" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="BH3" s="1" t="inlineStr">
-        <is>
-          <t>41000</t>
-        </is>
-      </c>
-      <c r="BI3" s="1" t="inlineStr">
-        <is>
-          <t>60500</t>
-        </is>
-      </c>
-      <c r="BJ3" s="1" t="inlineStr">
-        <is>
-          <t>11596</t>
-        </is>
-      </c>
-      <c r="BK3" s="1" t="inlineStr">
-        <is>
-          <t>Евро 5</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>